<commit_message>
updates on primary and secondary genes
1. updated primary and secondary genes' CpG sites

2. upload experimental data corresponding to primary and secondary CpG sites
</commit_message>
<xml_diff>
--- a/primary genes/primary gene and CPG.xlsx
+++ b/primary genes/primary gene and CPG.xlsx
@@ -351,7 +351,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B234"/>
+  <dimension ref="A1:C233"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -365,6 +365,11 @@
           <t>X.19</t>
         </is>
       </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -377,6 +382,9 @@
           <t>APLN</t>
         </is>
       </c>
+      <c r="C2">
+        <v>1</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -389,6 +397,9 @@
           <t>APLN</t>
         </is>
       </c>
+      <c r="C3">
+        <v>2</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -401,6 +412,9 @@
           <t>APLN</t>
         </is>
       </c>
+      <c r="C4">
+        <v>3</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -413,6 +427,9 @@
           <t>APLN</t>
         </is>
       </c>
+      <c r="C5">
+        <v>4</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -425,6 +442,9 @@
           <t>APLN</t>
         </is>
       </c>
+      <c r="C6">
+        <v>5</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -437,6 +457,9 @@
           <t>APLN</t>
         </is>
       </c>
+      <c r="C7">
+        <v>6</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -449,6 +472,9 @@
           <t>APLN;APLN</t>
         </is>
       </c>
+      <c r="C8">
+        <v>7</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -461,6 +487,9 @@
           <t>APLN</t>
         </is>
       </c>
+      <c r="C9">
+        <v>8</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -473,6 +502,9 @@
           <t>APLN</t>
         </is>
       </c>
+      <c r="C10">
+        <v>9</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -485,6 +517,9 @@
           <t>APLN</t>
         </is>
       </c>
+      <c r="C11">
+        <v>10</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -497,6 +532,9 @@
           <t>APLN;APLN</t>
         </is>
       </c>
+      <c r="C12">
+        <v>11</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -509,6 +547,9 @@
           <t>APLN</t>
         </is>
       </c>
+      <c r="C13">
+        <v>12</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -521,6 +562,9 @@
           <t>APLN</t>
         </is>
       </c>
+      <c r="C14">
+        <v>13</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -533,6 +577,9 @@
           <t>MMP12</t>
         </is>
       </c>
+      <c r="C15">
+        <v>14</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -545,6 +592,9 @@
           <t>MMP12</t>
         </is>
       </c>
+      <c r="C16">
+        <v>15</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -557,6 +607,9 @@
           <t>MMP12</t>
         </is>
       </c>
+      <c r="C17">
+        <v>16</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -569,6 +622,9 @@
           <t>MMP12</t>
         </is>
       </c>
+      <c r="C18">
+        <v>17</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -581,6 +637,9 @@
           <t>MMP12;MMP12</t>
         </is>
       </c>
+      <c r="C19">
+        <v>18</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -593,6 +652,9 @@
           <t>MMP12</t>
         </is>
       </c>
+      <c r="C20">
+        <v>19</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -605,6 +667,9 @@
           <t>NOS2</t>
         </is>
       </c>
+      <c r="C21">
+        <v>20</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -617,6 +682,9 @@
           <t>NOS2;NOS2</t>
         </is>
       </c>
+      <c r="C22">
+        <v>21</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -629,6 +697,9 @@
           <t>NOS2</t>
         </is>
       </c>
+      <c r="C23">
+        <v>22</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -641,6 +712,9 @@
           <t>NOS2</t>
         </is>
       </c>
+      <c r="C24">
+        <v>23</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -653,6 +727,9 @@
           <t>NOS2</t>
         </is>
       </c>
+      <c r="C25">
+        <v>24</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -665,6 +742,9 @@
           <t>NOS2</t>
         </is>
       </c>
+      <c r="C26">
+        <v>25</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -677,6 +757,9 @@
           <t>NOS2</t>
         </is>
       </c>
+      <c r="C27">
+        <v>26</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -689,6 +772,9 @@
           <t>NOS2;NOS2</t>
         </is>
       </c>
+      <c r="C28">
+        <v>27</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -701,6 +787,9 @@
           <t>NOS2;NOS2</t>
         </is>
       </c>
+      <c r="C29">
+        <v>28</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -713,6 +802,9 @@
           <t>NOS2;NOS2</t>
         </is>
       </c>
+      <c r="C30">
+        <v>29</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -725,6 +817,9 @@
           <t>NOS2</t>
         </is>
       </c>
+      <c r="C31">
+        <v>30</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -737,6 +832,9 @@
           <t>NOS2</t>
         </is>
       </c>
+      <c r="C32">
+        <v>31</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -749,6 +847,9 @@
           <t>NOS2</t>
         </is>
       </c>
+      <c r="C33">
+        <v>32</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -761,6 +862,9 @@
           <t>NOS2</t>
         </is>
       </c>
+      <c r="C34">
+        <v>33</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -773,6 +877,9 @@
           <t>NOS2</t>
         </is>
       </c>
+      <c r="C35">
+        <v>34</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -785,6 +892,9 @@
           <t>NOS2;NOS2</t>
         </is>
       </c>
+      <c r="C36">
+        <v>35</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -797,6 +907,9 @@
           <t>ARG1</t>
         </is>
       </c>
+      <c r="C37">
+        <v>36</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -809,6 +922,9 @@
           <t>ARG1</t>
         </is>
       </c>
+      <c r="C38">
+        <v>37</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -821,6 +937,9 @@
           <t>ARG1</t>
         </is>
       </c>
+      <c r="C39">
+        <v>38</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -833,6 +952,9 @@
           <t>ARG1</t>
         </is>
       </c>
+      <c r="C40">
+        <v>39</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -845,6 +967,9 @@
           <t>ARG1;MED23</t>
         </is>
       </c>
+      <c r="C41">
+        <v>40</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -857,6 +982,9 @@
           <t>ARG1;MED23</t>
         </is>
       </c>
+      <c r="C42">
+        <v>41</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -869,6 +997,9 @@
           <t>ARG2</t>
         </is>
       </c>
+      <c r="C43">
+        <v>42</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -881,6 +1012,9 @@
           <t>ARG2</t>
         </is>
       </c>
+      <c r="C44">
+        <v>43</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -893,6 +1027,9 @@
           <t>ARG2</t>
         </is>
       </c>
+      <c r="C45">
+        <v>44</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -905,6 +1042,9 @@
           <t>ARG2</t>
         </is>
       </c>
+      <c r="C46">
+        <v>45</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -917,6 +1057,9 @@
           <t>ARG2</t>
         </is>
       </c>
+      <c r="C47">
+        <v>46</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -929,6 +1072,9 @@
           <t>ARG2</t>
         </is>
       </c>
+      <c r="C48">
+        <v>47</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -941,6 +1087,9 @@
           <t>ARG2;ARG2</t>
         </is>
       </c>
+      <c r="C49">
+        <v>48</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -953,6 +1102,9 @@
           <t>ARG2</t>
         </is>
       </c>
+      <c r="C50">
+        <v>49</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -965,6 +1117,9 @@
           <t>ARG2</t>
         </is>
       </c>
+      <c r="C51">
+        <v>50</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -977,6 +1132,9 @@
           <t>ARG2</t>
         </is>
       </c>
+      <c r="C52">
+        <v>51</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -989,6 +1147,9 @@
           <t>ARG2</t>
         </is>
       </c>
+      <c r="C53">
+        <v>52</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -1001,6 +1162,9 @@
           <t>ARG2</t>
         </is>
       </c>
+      <c r="C54">
+        <v>53</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -1013,6 +1177,9 @@
           <t>ARG2</t>
         </is>
       </c>
+      <c r="C55">
+        <v>54</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -1025,6 +1192,9 @@
           <t>ARG2</t>
         </is>
       </c>
+      <c r="C56">
+        <v>55</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -1037,6 +1207,9 @@
           <t>ARG2</t>
         </is>
       </c>
+      <c r="C57">
+        <v>56</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -1049,6 +1222,9 @@
           <t>ARG2</t>
         </is>
       </c>
+      <c r="C58">
+        <v>57</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -1061,6 +1237,9 @@
           <t>TNF</t>
         </is>
       </c>
+      <c r="C59">
+        <v>58</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -1073,6 +1252,9 @@
           <t>TNF</t>
         </is>
       </c>
+      <c r="C60">
+        <v>59</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -1085,6 +1267,9 @@
           <t>TNF</t>
         </is>
       </c>
+      <c r="C61">
+        <v>60</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -1097,6 +1282,9 @@
           <t>TNF</t>
         </is>
       </c>
+      <c r="C62">
+        <v>61</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -1109,6 +1297,9 @@
           <t>TNF</t>
         </is>
       </c>
+      <c r="C63">
+        <v>62</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -1121,6 +1312,9 @@
           <t>TNF</t>
         </is>
       </c>
+      <c r="C64">
+        <v>63</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -1133,6 +1327,9 @@
           <t>TNF</t>
         </is>
       </c>
+      <c r="C65">
+        <v>64</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -1145,6 +1342,9 @@
           <t>TNF</t>
         </is>
       </c>
+      <c r="C66">
+        <v>65</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -1157,6 +1357,9 @@
           <t>TNF</t>
         </is>
       </c>
+      <c r="C67">
+        <v>66</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -1169,6 +1372,9 @@
           <t>TNF</t>
         </is>
       </c>
+      <c r="C68">
+        <v>67</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -1181,6 +1387,9 @@
           <t>TNF</t>
         </is>
       </c>
+      <c r="C69">
+        <v>68</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -1193,6 +1402,9 @@
           <t>TNF</t>
         </is>
       </c>
+      <c r="C70">
+        <v>69</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -1205,6 +1417,9 @@
           <t>TNF</t>
         </is>
       </c>
+      <c r="C71">
+        <v>70</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -1217,6 +1432,9 @@
           <t>TNF</t>
         </is>
       </c>
+      <c r="C72">
+        <v>71</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -1229,6 +1447,9 @@
           <t>TNF</t>
         </is>
       </c>
+      <c r="C73">
+        <v>72</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -1241,6 +1462,9 @@
           <t>TNF</t>
         </is>
       </c>
+      <c r="C74">
+        <v>73</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -1253,6 +1477,9 @@
           <t>TNF</t>
         </is>
       </c>
+      <c r="C75">
+        <v>74</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -1265,6 +1492,9 @@
           <t>TNF</t>
         </is>
       </c>
+      <c r="C76">
+        <v>75</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -1277,6 +1507,9 @@
           <t>TNF</t>
         </is>
       </c>
+      <c r="C77">
+        <v>76</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -1289,6 +1522,9 @@
           <t>TNF</t>
         </is>
       </c>
+      <c r="C78">
+        <v>77</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -1301,6 +1537,9 @@
           <t>TNF</t>
         </is>
       </c>
+      <c r="C79">
+        <v>78</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -1313,6 +1552,9 @@
           <t>TNF</t>
         </is>
       </c>
+      <c r="C80">
+        <v>79</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -1325,6 +1567,9 @@
           <t>TNF</t>
         </is>
       </c>
+      <c r="C81">
+        <v>80</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -1337,6 +1582,9 @@
           <t>TNF</t>
         </is>
       </c>
+      <c r="C82">
+        <v>81</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -1349,6 +1597,9 @@
           <t>TNF</t>
         </is>
       </c>
+      <c r="C83">
+        <v>82</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -1361,6 +1612,9 @@
           <t>TNF</t>
         </is>
       </c>
+      <c r="C84">
+        <v>83</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -1373,6 +1627,9 @@
           <t>TNF</t>
         </is>
       </c>
+      <c r="C85">
+        <v>84</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -1385,6 +1642,9 @@
           <t>ICAM1</t>
         </is>
       </c>
+      <c r="C86">
+        <v>85</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -1397,6 +1657,9 @@
           <t>ICAM1</t>
         </is>
       </c>
+      <c r="C87">
+        <v>86</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -1409,6 +1672,9 @@
           <t>ICAM1;ICAM1</t>
         </is>
       </c>
+      <c r="C88">
+        <v>87</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -1421,6 +1687,9 @@
           <t>ICAM1</t>
         </is>
       </c>
+      <c r="C89">
+        <v>88</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -1433,6 +1702,9 @@
           <t>ICAM1</t>
         </is>
       </c>
+      <c r="C90">
+        <v>89</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -1445,6 +1717,9 @@
           <t>ICAM1</t>
         </is>
       </c>
+      <c r="C91">
+        <v>90</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -1457,6 +1732,9 @@
           <t>ICAM1</t>
         </is>
       </c>
+      <c r="C92">
+        <v>91</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -1469,6 +1747,9 @@
           <t>ICAM1</t>
         </is>
       </c>
+      <c r="C93">
+        <v>92</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -1481,6 +1762,9 @@
           <t>ICAM1</t>
         </is>
       </c>
+      <c r="C94">
+        <v>93</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -1493,6 +1777,9 @@
           <t>ICAM1</t>
         </is>
       </c>
+      <c r="C95">
+        <v>94</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -1505,6 +1792,9 @@
           <t>ICAM1</t>
         </is>
       </c>
+      <c r="C96">
+        <v>95</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -1517,6 +1807,9 @@
           <t>ICAM1</t>
         </is>
       </c>
+      <c r="C97">
+        <v>96</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -1529,6 +1822,9 @@
           <t>ICAM1;ICAM1</t>
         </is>
       </c>
+      <c r="C98">
+        <v>97</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -1541,6 +1837,9 @@
           <t>ICAM1</t>
         </is>
       </c>
+      <c r="C99">
+        <v>98</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -1553,6 +1852,9 @@
           <t>ICAM1</t>
         </is>
       </c>
+      <c r="C100">
+        <v>99</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -1565,6 +1867,9 @@
           <t>ICAM1</t>
         </is>
       </c>
+      <c r="C101">
+        <v>100</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -1577,6 +1882,9 @@
           <t>GSTM1;GSTM1</t>
         </is>
       </c>
+      <c r="C102">
+        <v>101</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -1589,6 +1897,9 @@
           <t>GSTM1;GSTM1</t>
         </is>
       </c>
+      <c r="C103">
+        <v>102</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -1601,6 +1912,9 @@
           <t>GSTM1;GSTM1</t>
         </is>
       </c>
+      <c r="C104">
+        <v>103</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -1613,1535 +1927,1919 @@
           <t>GSTM1;GSTM1;GSTM1;GSTM1</t>
         </is>
       </c>
+      <c r="C105">
+        <v>104</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>cg18938907</t>
+          <t>cg23241950</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>GSTM1;GSTM1;GSTM1;GSTM1</t>
-        </is>
+          <t>GSTM1;GSTM1</t>
+        </is>
+      </c>
+      <c r="C106">
+        <v>105</v>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>cg23241950</t>
+          <t>cg24506221</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
           <t>GSTM1;GSTM1</t>
         </is>
+      </c>
+      <c r="C107">
+        <v>106</v>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>cg24506221</t>
+          <t>cg00000884</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>GSTM1;GSTM1</t>
-        </is>
+          <t>TLR2</t>
+        </is>
+      </c>
+      <c r="C108">
+        <v>107</v>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>cg00000884</t>
+          <t>cg01554777</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
           <t>TLR2</t>
         </is>
+      </c>
+      <c r="C109">
+        <v>108</v>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>cg01554777</t>
+          <t>cg03523945</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
           <t>TLR2</t>
         </is>
+      </c>
+      <c r="C110">
+        <v>109</v>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>cg03523945</t>
+          <t>cg03610073</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
           <t>TLR2</t>
         </is>
+      </c>
+      <c r="C111">
+        <v>110</v>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>cg03610073</t>
+          <t>cg06405222</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
           <t>TLR2</t>
         </is>
+      </c>
+      <c r="C112">
+        <v>111</v>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>cg06405222</t>
+          <t>cg06618866</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
           <t>TLR2</t>
         </is>
+      </c>
+      <c r="C113">
+        <v>112</v>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>cg06618866</t>
+          <t>cg09623286</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>TLR2</t>
-        </is>
+          <t>TLR2;TLR2</t>
+        </is>
+      </c>
+      <c r="C114">
+        <v>113</v>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>cg09623286</t>
+          <t>cg12940473</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>TLR2;TLR2</t>
-        </is>
+          <t>TLR2</t>
+        </is>
+      </c>
+      <c r="C115">
+        <v>114</v>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>cg12940473</t>
+          <t>cg15852258</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
           <t>TLR2</t>
         </is>
+      </c>
+      <c r="C116">
+        <v>115</v>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>cg15852258</t>
+          <t>cg16547110</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
           <t>TLR2</t>
         </is>
+      </c>
+      <c r="C117">
+        <v>116</v>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>cg16547110</t>
+          <t>cg18652319</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
           <t>TLR2</t>
         </is>
+      </c>
+      <c r="C118">
+        <v>117</v>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>cg18652319</t>
+          <t>cg19037167</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
           <t>TLR2</t>
         </is>
+      </c>
+      <c r="C119">
+        <v>118</v>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>cg19037167</t>
+          <t>cg00306510</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>TLR2</t>
-        </is>
+          <t>TLR3</t>
+        </is>
+      </c>
+      <c r="C120">
+        <v>119</v>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>cg00306510</t>
+          <t>cg06498520</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
           <t>TLR3</t>
         </is>
+      </c>
+      <c r="C121">
+        <v>120</v>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>cg06498520</t>
+          <t>cg12281049</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>TLR3</t>
-        </is>
+          <t>TLR3;TLR3</t>
+        </is>
+      </c>
+      <c r="C122">
+        <v>121</v>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>cg12281049</t>
+          <t>cg12697789</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>TLR3;TLR3</t>
-        </is>
+          <t>TLR3</t>
+        </is>
+      </c>
+      <c r="C123">
+        <v>122</v>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>cg12697789</t>
+          <t>cg12950492</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
           <t>TLR3</t>
         </is>
+      </c>
+      <c r="C124">
+        <v>123</v>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>cg12950492</t>
+          <t>cg14827929</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
         <is>
           <t>TLR3</t>
         </is>
+      </c>
+      <c r="C125">
+        <v>124</v>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>cg14827929</t>
+          <t>cg17671280</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
         <is>
           <t>TLR3</t>
         </is>
+      </c>
+      <c r="C126">
+        <v>125</v>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>cg17671280</t>
+          <t>cg25367691</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>TLR3</t>
-        </is>
+          <t>TLR3;TLR3</t>
+        </is>
+      </c>
+      <c r="C127">
+        <v>126</v>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>cg25367691</t>
+          <t>cg02515422</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>TLR3;TLR3</t>
-        </is>
+          <t>TLR4;TLR4;TLR4;TLR4</t>
+        </is>
+      </c>
+      <c r="C128">
+        <v>127</v>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>cg02515422</t>
+          <t>cg05429895</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
         <is>
           <t>TLR4;TLR4;TLR4;TLR4</t>
         </is>
+      </c>
+      <c r="C129">
+        <v>128</v>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>cg05429895</t>
+          <t>cg13730105</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>TLR4;TLR4;TLR4;TLR4</t>
-        </is>
+          <t>TLR4;TLR4;TLR4</t>
+        </is>
+      </c>
+      <c r="C130">
+        <v>129</v>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>cg13730105</t>
+          <t>cg14605396</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
         <is>
           <t>TLR4;TLR4;TLR4</t>
         </is>
+      </c>
+      <c r="C131">
+        <v>130</v>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>cg14605396</t>
+          <t>cg14629571</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
         <is>
           <t>TLR4;TLR4;TLR4</t>
         </is>
+      </c>
+      <c r="C132">
+        <v>131</v>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>cg14629571</t>
+          <t>cg00087425</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>TLR4;TLR4;TLR4</t>
-        </is>
+          <t>IL6;IL6</t>
+        </is>
+      </c>
+      <c r="C133">
+        <v>132</v>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>cg00087425</t>
+          <t>cg01770232</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>IL6;IL6</t>
-        </is>
+          <t>IL6</t>
+        </is>
+      </c>
+      <c r="C134">
+        <v>133</v>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>cg01770232</t>
+          <t>cg02335517</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
         <is>
           <t>IL6</t>
         </is>
+      </c>
+      <c r="C135">
+        <v>134</v>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>cg02335517</t>
+          <t>cg05265849</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
         <is>
           <t>IL6</t>
         </is>
+      </c>
+      <c r="C136">
+        <v>135</v>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>cg05265849</t>
+          <t>cg05472934</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
         <is>
           <t>IL6</t>
         </is>
+      </c>
+      <c r="C137">
+        <v>136</v>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>cg05472934</t>
+          <t>cg07998387</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
         <is>
           <t>IL6</t>
         </is>
+      </c>
+      <c r="C138">
+        <v>137</v>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>cg07998387</t>
+          <t>cg10140158</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
         <is>
           <t>IL6</t>
         </is>
+      </c>
+      <c r="C139">
+        <v>138</v>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>cg10140158</t>
+          <t>cg13104385</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
         <is>
           <t>IL6</t>
         </is>
+      </c>
+      <c r="C140">
+        <v>139</v>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>cg13104385</t>
+          <t>cg15703690</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
         <is>
           <t>IL6</t>
         </is>
+      </c>
+      <c r="C141">
+        <v>140</v>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>cg15703690</t>
+          <t>cg17067544</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
         <is>
           <t>IL6</t>
         </is>
+      </c>
+      <c r="C142">
+        <v>141</v>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>cg17067544</t>
+          <t>cg26061582</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
         <is>
           <t>IL6</t>
         </is>
+      </c>
+      <c r="C143">
+        <v>142</v>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>cg26061582</t>
+          <t>cg04392234</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>IL6</t>
-        </is>
+          <t>IL8</t>
+        </is>
+      </c>
+      <c r="C144">
+        <v>143</v>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>cg04392234</t>
+          <t>cg16468729</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
         <is>
           <t>IL8</t>
         </is>
+      </c>
+      <c r="C145">
+        <v>144</v>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>cg16468729</t>
+          <t>cg01290568</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>IL8</t>
-        </is>
+          <t>IL1B</t>
+        </is>
+      </c>
+      <c r="C146">
+        <v>145</v>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>cg01290568</t>
+          <t>cg02596281</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
         <is>
           <t>IL1B</t>
         </is>
+      </c>
+      <c r="C147">
+        <v>146</v>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>cg02596281</t>
+          <t>cg07935264</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
         <is>
           <t>IL1B</t>
         </is>
+      </c>
+      <c r="C148">
+        <v>147</v>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>cg07935264</t>
+          <t>cg14117934</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
         <is>
           <t>IL1B</t>
         </is>
+      </c>
+      <c r="C149">
+        <v>148</v>
       </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>cg14117934</t>
+          <t>cg15836722</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
         <is>
           <t>IL1B</t>
         </is>
+      </c>
+      <c r="C150">
+        <v>149</v>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>cg15836722</t>
+          <t>cg18635064</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
         <is>
           <t>IL1B</t>
         </is>
+      </c>
+      <c r="C151">
+        <v>150</v>
       </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>cg18635064</t>
+          <t>cg18773937</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
         <is>
           <t>IL1B</t>
         </is>
+      </c>
+      <c r="C152">
+        <v>151</v>
       </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>cg18773937</t>
+          <t>cg20157753</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>IL1B</t>
-        </is>
+          <t>IL1B;IL1B</t>
+        </is>
+      </c>
+      <c r="C153">
+        <v>152</v>
       </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>cg20157753</t>
+          <t>cg23149881</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>IL1B;IL1B</t>
-        </is>
+          <t>IL1B</t>
+        </is>
+      </c>
+      <c r="C154">
+        <v>153</v>
       </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>cg23149881</t>
+          <t>cg00447324</t>
         </is>
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>IL1B</t>
-        </is>
+          <t>CCL5</t>
+        </is>
+      </c>
+      <c r="C155">
+        <v>154</v>
       </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>cg00447324</t>
+          <t>cg02483931</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
         <is>
           <t>CCL5</t>
         </is>
+      </c>
+      <c r="C156">
+        <v>155</v>
       </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>cg02483931</t>
+          <t>cg02867514</t>
         </is>
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>CCL5</t>
-        </is>
+          <t>CCL5;CCL5</t>
+        </is>
+      </c>
+      <c r="C157">
+        <v>156</v>
       </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>cg02867514</t>
+          <t>cg04791421</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>CCL5;CCL5</t>
-        </is>
+          <t>CCL5</t>
+        </is>
+      </c>
+      <c r="C158">
+        <v>157</v>
       </c>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>cg04791421</t>
+          <t>cg08656816</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
         <is>
           <t>CCL5</t>
         </is>
+      </c>
+      <c r="C159">
+        <v>158</v>
       </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>cg08656816</t>
+          <t>cg10315334</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>CCL5</t>
-        </is>
+          <t>CCL5;CCL5</t>
+        </is>
+      </c>
+      <c r="C160">
+        <v>159</v>
       </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>cg10315334</t>
+          <t>cg12455187</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>CCL5;CCL5</t>
-        </is>
+          <t>CCL5</t>
+        </is>
+      </c>
+      <c r="C161">
+        <v>160</v>
       </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>cg12455187</t>
+          <t>cg14796318</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
         <is>
           <t>CCL5</t>
         </is>
+      </c>
+      <c r="C162">
+        <v>161</v>
       </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>cg14796318</t>
+          <t>cg19411729</t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
         <is>
           <t>CCL5</t>
         </is>
+      </c>
+      <c r="C163">
+        <v>162</v>
       </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>cg19411729</t>
+          <t>cg03812679</t>
         </is>
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>CCL5</t>
-        </is>
+          <t>CSF3;CSF3;CSF3</t>
+        </is>
+      </c>
+      <c r="C164">
+        <v>163</v>
       </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>cg03812679</t>
+          <t>cg04193923</t>
         </is>
       </c>
       <c r="B165" t="inlineStr">
         <is>
           <t>CSF3;CSF3;CSF3</t>
         </is>
+      </c>
+      <c r="C165">
+        <v>164</v>
       </c>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>cg04193923</t>
+          <t>cg07472953</t>
         </is>
       </c>
       <c r="B166" t="inlineStr">
         <is>
           <t>CSF3;CSF3;CSF3</t>
         </is>
+      </c>
+      <c r="C166">
+        <v>165</v>
       </c>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>cg07472953</t>
+          <t>cg07584981</t>
         </is>
       </c>
       <c r="B167" t="inlineStr">
         <is>
           <t>CSF3;CSF3;CSF3</t>
         </is>
+      </c>
+      <c r="C167">
+        <v>166</v>
       </c>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>cg07584981</t>
+          <t>cg09161579</t>
         </is>
       </c>
       <c r="B168" t="inlineStr">
         <is>
           <t>CSF3;CSF3;CSF3</t>
         </is>
+      </c>
+      <c r="C168">
+        <v>167</v>
       </c>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>cg09161579</t>
+          <t>cg16271663</t>
         </is>
       </c>
       <c r="B169" t="inlineStr">
         <is>
           <t>CSF3;CSF3;CSF3</t>
         </is>
+      </c>
+      <c r="C169">
+        <v>168</v>
       </c>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>cg16271663</t>
+          <t>cg21432842</t>
         </is>
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>CSF3;CSF3;CSF3</t>
-        </is>
+          <t>CSF3;CSF3;CSF3;CSF3;CSF3;CSF3</t>
+        </is>
+      </c>
+      <c r="C170">
+        <v>169</v>
       </c>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>cg21432842</t>
+          <t>cg23207054</t>
         </is>
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>CSF3;CSF3;CSF3;CSF3;CSF3;CSF3</t>
-        </is>
+          <t>CSF3;CSF3;CSF3</t>
+        </is>
+      </c>
+      <c r="C171">
+        <v>170</v>
       </c>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>cg23207054</t>
+          <t>cg02196805</t>
         </is>
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>CSF3;CSF3;CSF3</t>
-        </is>
+          <t>CSF2</t>
+        </is>
+      </c>
+      <c r="C172">
+        <v>171</v>
       </c>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>cg02196805</t>
+          <t>cg02325250</t>
         </is>
       </c>
       <c r="B173" t="inlineStr">
         <is>
           <t>CSF2</t>
         </is>
+      </c>
+      <c r="C173">
+        <v>172</v>
       </c>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>cg02325250</t>
+          <t>cg08324925</t>
         </is>
       </c>
       <c r="B174" t="inlineStr">
         <is>
           <t>CSF2</t>
         </is>
+      </c>
+      <c r="C174">
+        <v>173</v>
       </c>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>cg08324925</t>
+          <t>cg08686879</t>
         </is>
       </c>
       <c r="B175" t="inlineStr">
         <is>
           <t>CSF2</t>
         </is>
+      </c>
+      <c r="C175">
+        <v>174</v>
       </c>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>cg08686879</t>
+          <t>cg13259290</t>
         </is>
       </c>
       <c r="B176" t="inlineStr">
         <is>
           <t>CSF2</t>
         </is>
+      </c>
+      <c r="C176">
+        <v>175</v>
       </c>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>cg13259290</t>
+          <t>cg14675871</t>
         </is>
       </c>
       <c r="B177" t="inlineStr">
         <is>
           <t>CSF2</t>
         </is>
+      </c>
+      <c r="C177">
+        <v>176</v>
       </c>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>cg14675871</t>
+          <t>cg16465129</t>
         </is>
       </c>
       <c r="B178" t="inlineStr">
         <is>
           <t>CSF2</t>
         </is>
+      </c>
+      <c r="C178">
+        <v>177</v>
       </c>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>cg16465129</t>
+          <t>cg16565692</t>
         </is>
       </c>
       <c r="B179" t="inlineStr">
         <is>
           <t>CSF2</t>
         </is>
+      </c>
+      <c r="C179">
+        <v>178</v>
       </c>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>cg16565692</t>
+          <t>cg17566874</t>
         </is>
       </c>
       <c r="B180" t="inlineStr">
         <is>
           <t>CSF2</t>
         </is>
+      </c>
+      <c r="C180">
+        <v>179</v>
       </c>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>cg17566874</t>
+          <t>cg20704330</t>
         </is>
       </c>
       <c r="B181" t="inlineStr">
         <is>
           <t>CSF2</t>
         </is>
+      </c>
+      <c r="C181">
+        <v>180</v>
       </c>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>cg20704330</t>
+          <t>cg26369418</t>
         </is>
       </c>
       <c r="B182" t="inlineStr">
         <is>
           <t>CSF2</t>
         </is>
+      </c>
+      <c r="C182">
+        <v>181</v>
       </c>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>cg26369418</t>
+          <t>cg00524486</t>
         </is>
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>CSF2</t>
-        </is>
+          <t>MUC5B</t>
+        </is>
+      </c>
+      <c r="C183">
+        <v>182</v>
       </c>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>cg00524486</t>
+          <t>cg01133890</t>
         </is>
       </c>
       <c r="B184" t="inlineStr">
         <is>
           <t>MUC5B</t>
         </is>
+      </c>
+      <c r="C184">
+        <v>183</v>
       </c>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>cg01133890</t>
+          <t>cg01236384</t>
         </is>
       </c>
       <c r="B185" t="inlineStr">
         <is>
           <t>MUC5B</t>
         </is>
+      </c>
+      <c r="C185">
+        <v>184</v>
       </c>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>cg01236384</t>
+          <t>cg01264919</t>
         </is>
       </c>
       <c r="B186" t="inlineStr">
         <is>
           <t>MUC5B</t>
         </is>
+      </c>
+      <c r="C186">
+        <v>185</v>
       </c>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>cg01264919</t>
+          <t>cg01554231</t>
         </is>
       </c>
       <c r="B187" t="inlineStr">
         <is>
           <t>MUC5B</t>
         </is>
+      </c>
+      <c r="C187">
+        <v>186</v>
       </c>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>cg01554231</t>
+          <t>cg01989504</t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
         <is>
           <t>MUC5B</t>
         </is>
+      </c>
+      <c r="C188">
+        <v>187</v>
       </c>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>cg01989504</t>
+          <t>cg02379155</t>
         </is>
       </c>
       <c r="B189" t="inlineStr">
         <is>
           <t>MUC5B</t>
         </is>
+      </c>
+      <c r="C189">
+        <v>188</v>
       </c>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>cg02379155</t>
+          <t>cg02522041</t>
         </is>
       </c>
       <c r="B190" t="inlineStr">
         <is>
           <t>MUC5B</t>
         </is>
+      </c>
+      <c r="C190">
+        <v>189</v>
       </c>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>cg02522041</t>
+          <t>cg02680732</t>
         </is>
       </c>
       <c r="B191" t="inlineStr">
         <is>
           <t>MUC5B</t>
         </is>
+      </c>
+      <c r="C191">
+        <v>190</v>
       </c>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>cg02680732</t>
+          <t>cg03609102</t>
         </is>
       </c>
       <c r="B192" t="inlineStr">
         <is>
           <t>MUC5B</t>
         </is>
+      </c>
+      <c r="C192">
+        <v>191</v>
       </c>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>cg03609102</t>
+          <t>cg04449523</t>
         </is>
       </c>
       <c r="B193" t="inlineStr">
         <is>
           <t>MUC5B</t>
         </is>
+      </c>
+      <c r="C193">
+        <v>192</v>
       </c>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>cg04449523</t>
+          <t>cg00294956</t>
         </is>
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>MUC5B</t>
-        </is>
+          <t>DNAH5</t>
+        </is>
+      </c>
+      <c r="C194">
+        <v>193</v>
       </c>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>cg00294956</t>
+          <t>cg00600661</t>
         </is>
       </c>
       <c r="B195" t="inlineStr">
         <is>
           <t>DNAH5</t>
         </is>
+      </c>
+      <c r="C195">
+        <v>194</v>
       </c>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>cg00600661</t>
+          <t>cg03503295</t>
         </is>
       </c>
       <c r="B196" t="inlineStr">
         <is>
           <t>DNAH5</t>
         </is>
+      </c>
+      <c r="C196">
+        <v>195</v>
       </c>
     </row>
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>cg03503295</t>
+          <t>cg04192593</t>
         </is>
       </c>
       <c r="B197" t="inlineStr">
         <is>
           <t>DNAH5</t>
         </is>
+      </c>
+      <c r="C197">
+        <v>196</v>
       </c>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>cg04192593</t>
+          <t>cg04734587</t>
         </is>
       </c>
       <c r="B198" t="inlineStr">
         <is>
           <t>DNAH5</t>
         </is>
+      </c>
+      <c r="C198">
+        <v>197</v>
       </c>
     </row>
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>cg04734587</t>
+          <t>cg05004705</t>
         </is>
       </c>
       <c r="B199" t="inlineStr">
         <is>
           <t>DNAH5</t>
         </is>
+      </c>
+      <c r="C199">
+        <v>198</v>
       </c>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>cg05004705</t>
+          <t>cg05149258</t>
         </is>
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>DNAH5</t>
-        </is>
+          <t>DNAH5;DNAH5</t>
+        </is>
+      </c>
+      <c r="C200">
+        <v>199</v>
       </c>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>cg05149258</t>
+          <t>cg07548982</t>
         </is>
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>DNAH5;DNAH5</t>
-        </is>
+          <t>DNAH5</t>
+        </is>
+      </c>
+      <c r="C201">
+        <v>200</v>
       </c>
     </row>
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>cg07548982</t>
+          <t>cg07563943</t>
         </is>
       </c>
       <c r="B202" t="inlineStr">
         <is>
           <t>DNAH5</t>
         </is>
+      </c>
+      <c r="C202">
+        <v>201</v>
       </c>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>cg07563943</t>
+          <t>cg08442052</t>
         </is>
       </c>
       <c r="B203" t="inlineStr">
         <is>
           <t>DNAH5</t>
         </is>
+      </c>
+      <c r="C203">
+        <v>202</v>
       </c>
     </row>
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>cg08442052</t>
+          <t>cg08818829</t>
         </is>
       </c>
       <c r="B204" t="inlineStr">
         <is>
           <t>DNAH5</t>
         </is>
+      </c>
+      <c r="C204">
+        <v>203</v>
       </c>
     </row>
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>cg08818829</t>
+          <t>cg13896699</t>
         </is>
       </c>
       <c r="B205" t="inlineStr">
         <is>
           <t>DNAH5</t>
         </is>
+      </c>
+      <c r="C205">
+        <v>204</v>
       </c>
     </row>
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>cg13896699</t>
+          <t>cg14880800</t>
         </is>
       </c>
       <c r="B206" t="inlineStr">
         <is>
           <t>DNAH5</t>
         </is>
+      </c>
+      <c r="C206">
+        <v>205</v>
       </c>
     </row>
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>cg14880800</t>
+          <t>cg15416770</t>
         </is>
       </c>
       <c r="B207" t="inlineStr">
         <is>
           <t>DNAH5</t>
         </is>
+      </c>
+      <c r="C207">
+        <v>206</v>
       </c>
     </row>
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>cg15416770</t>
+          <t>cg16403725</t>
         </is>
       </c>
       <c r="B208" t="inlineStr">
         <is>
           <t>DNAH5</t>
         </is>
+      </c>
+      <c r="C208">
+        <v>207</v>
       </c>
     </row>
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>cg16403725</t>
+          <t>cg18118535</t>
         </is>
       </c>
       <c r="B209" t="inlineStr">
         <is>
           <t>DNAH5</t>
         </is>
+      </c>
+      <c r="C209">
+        <v>208</v>
       </c>
     </row>
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>cg18118535</t>
+          <t>cg19540371</t>
         </is>
       </c>
       <c r="B210" t="inlineStr">
         <is>
           <t>DNAH5</t>
         </is>
+      </c>
+      <c r="C210">
+        <v>209</v>
       </c>
     </row>
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>cg19540371</t>
+          <t>cg20380465</t>
         </is>
       </c>
       <c r="B211" t="inlineStr">
         <is>
           <t>DNAH5</t>
         </is>
+      </c>
+      <c r="C211">
+        <v>210</v>
       </c>
     </row>
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>cg20380465</t>
+          <t>cg20738735</t>
         </is>
       </c>
       <c r="B212" t="inlineStr">
         <is>
           <t>DNAH5</t>
         </is>
+      </c>
+      <c r="C212">
+        <v>211</v>
       </c>
     </row>
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>cg20738735</t>
+          <t>cg22466716</t>
         </is>
       </c>
       <c r="B213" t="inlineStr">
         <is>
           <t>DNAH5</t>
         </is>
+      </c>
+      <c r="C213">
+        <v>212</v>
       </c>
     </row>
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>cg22466716</t>
+          <t>cg23504924</t>
         </is>
       </c>
       <c r="B214" t="inlineStr">
         <is>
           <t>DNAH5</t>
         </is>
+      </c>
+      <c r="C214">
+        <v>213</v>
       </c>
     </row>
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>cg23504924</t>
+          <t>cg26676090</t>
         </is>
       </c>
       <c r="B215" t="inlineStr">
         <is>
           <t>DNAH5</t>
         </is>
+      </c>
+      <c r="C215">
+        <v>214</v>
       </c>
     </row>
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>cg26676090</t>
+          <t>cg26992949</t>
         </is>
       </c>
       <c r="B216" t="inlineStr">
         <is>
           <t>DNAH5</t>
         </is>
+      </c>
+      <c r="C216">
+        <v>215</v>
       </c>
     </row>
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>cg26992949</t>
+          <t>cg00690431</t>
         </is>
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>DNAH5</t>
-        </is>
+          <t>PTGS2</t>
+        </is>
+      </c>
+      <c r="C217">
+        <v>216</v>
       </c>
     </row>
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>cg00690431</t>
+          <t>cg04881125</t>
         </is>
       </c>
       <c r="B218" t="inlineStr">
         <is>
           <t>PTGS2</t>
         </is>
+      </c>
+      <c r="C218">
+        <v>217</v>
       </c>
     </row>
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>cg04881125</t>
+          <t>cg07422329</t>
         </is>
       </c>
       <c r="B219" t="inlineStr">
         <is>
           <t>PTGS2</t>
         </is>
+      </c>
+      <c r="C219">
+        <v>218</v>
       </c>
     </row>
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>cg07422329</t>
+          <t>cg08482694</t>
         </is>
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>PTGS2</t>
-        </is>
+          <t>PTGS2;PTGS2</t>
+        </is>
+      </c>
+      <c r="C220">
+        <v>219</v>
       </c>
     </row>
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>cg08482694</t>
+          <t>cg09461185</t>
         </is>
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>PTGS2;PTGS2</t>
-        </is>
+          <t>PTGS2</t>
+        </is>
+      </c>
+      <c r="C221">
+        <v>220</v>
       </c>
     </row>
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>cg09461185</t>
+          <t>cg10180406</t>
         </is>
       </c>
       <c r="B222" t="inlineStr">
         <is>
           <t>PTGS2</t>
         </is>
+      </c>
+      <c r="C222">
+        <v>221</v>
       </c>
     </row>
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>cg10180406</t>
+          <t>cg13986130</t>
         </is>
       </c>
       <c r="B223" t="inlineStr">
         <is>
           <t>PTGS2</t>
         </is>
+      </c>
+      <c r="C223">
+        <v>222</v>
       </c>
     </row>
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>cg13986130</t>
+          <t>cg16101346</t>
         </is>
       </c>
       <c r="B224" t="inlineStr">
         <is>
           <t>PTGS2</t>
         </is>
+      </c>
+      <c r="C224">
+        <v>223</v>
       </c>
     </row>
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>cg16101346</t>
+          <t>cg17419623</t>
         </is>
       </c>
       <c r="B225" t="inlineStr">
         <is>
           <t>PTGS2</t>
         </is>
+      </c>
+      <c r="C225">
+        <v>224</v>
       </c>
     </row>
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>cg17419623</t>
+          <t>cg18335243</t>
         </is>
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>PTGS2</t>
-        </is>
+          <t>PTGS2;PTGS2</t>
+        </is>
+      </c>
+      <c r="C226">
+        <v>225</v>
       </c>
     </row>
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>cg18335243</t>
+          <t>cg19155599</t>
         </is>
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>PTGS2;PTGS2</t>
-        </is>
+          <t>PTGS2</t>
+        </is>
+      </c>
+      <c r="C227">
+        <v>226</v>
       </c>
     </row>
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>cg19155599</t>
+          <t>cg22365834</t>
         </is>
       </c>
       <c r="B228" t="inlineStr">
         <is>
           <t>PTGS2</t>
         </is>
+      </c>
+      <c r="C228">
+        <v>227</v>
       </c>
     </row>
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>cg22365834</t>
+          <t>cg23070111</t>
         </is>
       </c>
       <c r="B229" t="inlineStr">
         <is>
           <t>PTGS2</t>
         </is>
+      </c>
+      <c r="C229">
+        <v>228</v>
       </c>
     </row>
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>cg23070111</t>
+          <t>cg24887140</t>
         </is>
       </c>
       <c r="B230" t="inlineStr">
         <is>
           <t>PTGS2</t>
         </is>
+      </c>
+      <c r="C230">
+        <v>229</v>
       </c>
     </row>
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>cg24887140</t>
+          <t>cg25147026</t>
         </is>
       </c>
       <c r="B231" t="inlineStr">
         <is>
           <t>PTGS2</t>
         </is>
+      </c>
+      <c r="C231">
+        <v>230</v>
       </c>
     </row>
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>cg25147026</t>
+          <t>cg25837803</t>
         </is>
       </c>
       <c r="B232" t="inlineStr">
         <is>
           <t>PTGS2</t>
         </is>
+      </c>
+      <c r="C232">
+        <v>231</v>
       </c>
     </row>
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>cg25837803</t>
+          <t>cg26564040</t>
         </is>
       </c>
       <c r="B233" t="inlineStr">
@@ -3149,17 +3847,8 @@
           <t>PTGS2</t>
         </is>
       </c>
-    </row>
-    <row r="234">
-      <c r="A234" t="inlineStr">
-        <is>
-          <t>cg26564040</t>
-        </is>
-      </c>
-      <c r="B234" t="inlineStr">
-        <is>
-          <t>PTGS2</t>
-        </is>
+      <c r="C233">
+        <v>232</v>
       </c>
     </row>
   </sheetData>

</xml_diff>